<commit_message>
feat: prioritize new and changed reconciliation tasks while preserving review history
</commit_message>
<xml_diff>
--- a/examples/月末客户对账/复核工作簿.xlsx
+++ b/examples/月末客户对账/复核工作簿.xlsx
@@ -8,15 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待处理" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已匹配" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史记录" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="本次重点" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待处理" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="已匹配" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史记录" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_meta" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'待处理'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'已匹配'!$A$1:$L$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'历史记录'!$A$1:$L$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'本次重点'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'待处理'!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'已匹配'!$A$1:$L$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'历史记录'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +43,13 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -75,10 +84,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -90,12 +100,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -458,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -473,7 +485,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>0.7.0</t>
+          <t>0.8.0</t>
         </is>
       </c>
     </row>
@@ -525,7 +537,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>打开待处理页；优先看需重新复核和新增条目，在黄色列填写状态和意见。</t>
+          <t>先看本次重点，点击处理入口到待处理页填写黄色列；未变化但未解决的事项仍在跟进清单。</t>
         </is>
       </c>
     </row>
@@ -660,70 +672,122 @@
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>一致</t>
+          <t>本次重点</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>金额差异</t>
+          <t>旧事项仍待跟进</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>仅左表</t>
+          <t>已解决沿用</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>重复编号</t>
+          <t>上次记录本次未出现</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>无效金额</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>1</v>
+          <t>意见填写位置</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>只在待处理或已匹配页填写；本次重点为只读视图，避免两处意见不一致。</t>
+        </is>
       </c>
     </row>
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>仅右表</t>
+          <t>一致</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>金额差异</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>仅左表</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>重复编号</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>无效金额</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>仅右表</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>首次核对</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -733,6 +797,290 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>编号 / 联合键</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>核对结果</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>本次变化</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>处理状态</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>上次处理意见</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>左表原金额</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>右表原金额</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>左减右差额</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>处理入口</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SH-002</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>金额差异</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>首次核对</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2350.00</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2300.00</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>填写状态与意见</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SH-004</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>仅左表</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>首次核对</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>填写状态与意见</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SH-005</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>重复编号</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>首次核对</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>450.00 / 450.00</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>450.00</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>填写状态与意见</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SH-006</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>无效金额</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>首次核对</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>900.00</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>填写状态与意见</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SH-008</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>仅右表</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>首次核对</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待处理</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>600.00</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>填写状态与意见</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <autoFilter ref="A1:I6"/>
+  <hyperlinks>
+    <hyperlink ref="I2" location="'待处理'!D2" display="填写状态与意见"/>
+    <hyperlink ref="I3" location="'待处理'!D3" display="填写状态与意见"/>
+    <hyperlink ref="I4" location="'待处理'!D4" display="填写状态与意见"/>
+    <hyperlink ref="I5" location="'待处理'!D5" display="填写状态与意见"/>
+    <hyperlink ref="I6" location="'待处理'!D6" display="填写状态与意见"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -833,12 +1181,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>3</t>
@@ -891,12 +1239,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>5</t>
@@ -941,12 +1289,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>6 / 7</t>
@@ -999,12 +1347,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>8</t>
@@ -1053,12 +1401,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>待处理</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -1098,7 +1446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1199,12 +1547,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>无需处理</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>2</t>
@@ -1257,12 +1605,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>无需处理</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>4</t>
@@ -1315,12 +1663,12 @@
           <t>首次核对</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>无需处理</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>9</t>
@@ -1368,7 +1716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1459,7 +1807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>